<commit_message>
fixed the update window
</commit_message>
<xml_diff>
--- a/data/mappings.xlsx
+++ b/data/mappings.xlsx
@@ -1168,7 +1168,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>S:/DEV/Report-Generator/Rapport_data.xlsx</t>
+          <t>S:/DEV/Report-Generator/data/Rapport_data.xlsx</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>S:/DEV/Report-Generator/rapport_template.docx</t>
+          <t>S:/DEV/Report-Generator/data/rapport_template.docx</t>
         </is>
       </c>
     </row>

</xml_diff>